<commit_message>
Increase monster count, add stenball and lightning ball icon
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#MilestoneParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#MilestoneParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA39B26-EF7C-48D5-BE5F-7E0B9DF2214E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6169A1-2239-468E-AF59-9B163DCFA05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -649,7 +649,7 @@
         <v>1</v>
       </c>
       <c r="J5" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5" s="4">
         <v>5</v>
@@ -695,7 +695,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4">
         <v>6</v>
@@ -740,7 +740,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7" s="4">
         <v>7</v>
@@ -785,7 +785,7 @@
         <v>1.5</v>
       </c>
       <c r="J8" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4">
         <v>8</v>
@@ -830,7 +830,7 @@
         <v>1.5</v>
       </c>
       <c r="J9" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L9" s="1">
         <v>9</v>
@@ -875,7 +875,7 @@
         <v>1.5</v>
       </c>
       <c r="J10" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="1">
         <v>10</v>
@@ -920,7 +920,7 @@
         <v>1.5</v>
       </c>
       <c r="J11" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11" s="1">
         <v>11</v>
@@ -966,7 +966,7 @@
         <v>1.5</v>
       </c>
       <c r="J12" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12" s="1">
         <v>12</v>
@@ -1013,7 +1013,7 @@
         <v>1.5</v>
       </c>
       <c r="J13" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L13" s="1">
         <v>13</v>
@@ -1060,7 +1060,7 @@
         <v>2</v>
       </c>
       <c r="J14" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L14" s="1">
         <v>14</v>
@@ -1107,7 +1107,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L15" s="1">
         <v>15</v>
@@ -1154,7 +1154,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L16" s="1">
         <v>16</v>

</xml_diff>

<commit_message>
increase base point requirement
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#MilestoneParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#MilestoneParam.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6169A1-2239-468E-AF59-9B163DCFA05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D3BD39-2C44-4D3D-BC55-FB099BDC72E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -631,7 +631,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>9000</v>
+        <v>30000</v>
       </c>
       <c r="E5" s="1">
         <v>3</v>

</xml_diff>